<commit_message>
fix: main.py data acquisition
</commit_message>
<xml_diff>
--- a/reports/relatorio_investimento.xlsx
+++ b/reports/relatorio_investimento.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -514,37 +514,37 @@
         <v>0.9977540622750996</v>
       </c>
       <c r="C2" t="n">
-        <v>3.524412195831653</v>
+        <v>3.523123972571357</v>
       </c>
       <c r="D2" t="n">
-        <v>912551371.7137746</v>
+        <v>936702989.6828333</v>
       </c>
       <c r="E2" t="n">
-        <v>1.777495030877855e-11</v>
+        <v>1.602628234031397e-11</v>
       </c>
       <c r="F2" t="n">
-        <v>35.71428571428571</v>
+        <v>80</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3070159486932991</v>
+        <v>0.3082365131172478</v>
       </c>
       <c r="H2" t="n">
         <v>0.2864134091531322</v>
       </c>
       <c r="I2" t="n">
-        <v>57.14285714285714</v>
+        <v>45</v>
       </c>
       <c r="J2" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="K2" t="n">
-        <v>35.71428571428571</v>
+        <v>80</v>
       </c>
       <c r="L2" t="n">
-        <v>42.85714285714286</v>
+        <v>55</v>
       </c>
       <c r="M2" t="n">
-        <v>63.57142857142857</v>
+        <v>78.5</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -555,44 +555,44 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>VALE3</t>
+          <t>NEOE3</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.8207620043812851</v>
+        <v>0.7674675202273207</v>
       </c>
       <c r="C3" t="n">
-        <v>3.326412780089652</v>
+        <v>3.430425306946491</v>
       </c>
       <c r="D3" t="n">
-        <v>2398868387.076423</v>
+        <v>55593558.19838388</v>
       </c>
       <c r="E3" t="n">
-        <v>7.647041598128165e-12</v>
+        <v>2.730831357123434e-11</v>
       </c>
       <c r="F3" t="n">
-        <v>78.57142857142857</v>
+        <v>35</v>
       </c>
       <c r="G3" t="n">
-        <v>0.3567095385327261</v>
+        <v>0.01860445309896535</v>
       </c>
       <c r="H3" t="n">
-        <v>0.2543366296571614</v>
+        <v>0.02885617245514972</v>
       </c>
       <c r="I3" t="n">
-        <v>85.71428571428571</v>
+        <v>5</v>
       </c>
       <c r="J3" t="n">
-        <v>85.71428571428571</v>
+        <v>90</v>
       </c>
       <c r="K3" t="n">
-        <v>78.57142857142857</v>
+        <v>35</v>
       </c>
       <c r="L3" t="n">
-        <v>14.28571428571429</v>
+        <v>95</v>
       </c>
       <c r="M3" t="n">
-        <v>62.14285714285714</v>
+        <v>75</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -603,48 +603,48 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>VALE3</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.002795726117860386</v>
+        <v>0.8207620043812851</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.01056761352176577</v>
+        <v>3.315576634856987</v>
       </c>
       <c r="D4" t="n">
-        <v>14768618124.3547</v>
+        <v>2462520192.389824</v>
       </c>
       <c r="E4" t="n">
-        <v>7.794816665266045e-13</v>
+        <v>7.219603890928269e-12</v>
       </c>
       <c r="F4" t="n">
-        <v>92.85714285714286</v>
+        <v>97.5</v>
       </c>
       <c r="G4" t="n">
-        <v>0.2541466886367213</v>
+        <v>0.3639053817002734</v>
       </c>
       <c r="H4" t="n">
-        <v>0.2151546327929952</v>
+        <v>0.2579701008656878</v>
       </c>
       <c r="I4" t="n">
-        <v>14.28571428571428</v>
+        <v>65</v>
       </c>
       <c r="J4" t="n">
-        <v>14.28571428571428</v>
+        <v>85</v>
       </c>
       <c r="K4" t="n">
-        <v>92.85714285714286</v>
+        <v>97.5</v>
       </c>
       <c r="L4" t="n">
-        <v>85.71428571428572</v>
+        <v>35</v>
       </c>
       <c r="M4" t="n">
-        <v>59.28571428571428</v>
+        <v>73.75</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>NEUTRO</t>
+          <t>COMPRA MODERADA</t>
         </is>
       </c>
     </row>
@@ -658,41 +658,41 @@
         <v>0.6897098437509033</v>
       </c>
       <c r="C5" t="n">
-        <v>3.147924644483759</v>
+        <v>3.142741731706303</v>
       </c>
       <c r="D5" t="n">
-        <v>1686611723.969523</v>
+        <v>1720748464.992015</v>
       </c>
       <c r="E5" t="n">
-        <v>1.00673188090829e-11</v>
+        <v>9.931335673099017e-12</v>
       </c>
       <c r="F5" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.3283468072948462</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.2524664077859532</v>
+      </c>
+      <c r="I5" t="n">
         <v>50</v>
       </c>
-      <c r="G5" t="n">
-        <v>0.3252733872921393</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.2523599946119469</v>
-      </c>
-      <c r="I5" t="n">
-        <v>71.42857142857143</v>
-      </c>
       <c r="J5" t="n">
-        <v>71.42857142857143</v>
+        <v>80</v>
       </c>
       <c r="K5" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="L5" t="n">
         <v>50</v>
       </c>
-      <c r="L5" t="n">
-        <v>28.57142857142857</v>
-      </c>
       <c r="M5" t="n">
-        <v>52.14285714285714</v>
+        <v>73.25</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>NEUTRO</t>
+          <t>COMPRA MODERADA</t>
         </is>
       </c>
     </row>
@@ -706,41 +706,41 @@
         <v>0.3611223549013032</v>
       </c>
       <c r="C6" t="n">
-        <v>1.694658525640141</v>
+        <v>1.69311549253637</v>
       </c>
       <c r="D6" t="n">
-        <v>444647890.4039565</v>
+        <v>451478543.6449369</v>
       </c>
       <c r="E6" t="n">
-        <v>2.519363398876523e-11</v>
+        <v>2.610922385939225e-11</v>
       </c>
       <c r="F6" t="n">
-        <v>14.28571428571429</v>
+        <v>65</v>
       </c>
       <c r="G6" t="n">
-        <v>0.260145169409522</v>
+        <v>0.2621068729596222</v>
       </c>
       <c r="H6" t="n">
-        <v>0.2301036255099778</v>
+        <v>0.2309923257263864</v>
       </c>
       <c r="I6" t="n">
-        <v>28.57142857142857</v>
+        <v>10</v>
       </c>
       <c r="J6" t="n">
-        <v>57.14285714285714</v>
+        <v>65</v>
       </c>
       <c r="K6" t="n">
-        <v>14.28571428571429</v>
+        <v>65</v>
       </c>
       <c r="L6" t="n">
-        <v>71.42857142857143</v>
+        <v>90</v>
       </c>
       <c r="M6" t="n">
-        <v>48.57142857142857</v>
+        <v>72.5</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>NEUTRO</t>
+          <t>COMPRA MODERADA</t>
         </is>
       </c>
     </row>
@@ -751,92 +751,716 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.2069384299168635</v>
+        <v>0.2069382818126475</v>
       </c>
       <c r="C7" t="n">
-        <v>0.8486515303908404</v>
+        <v>0.8539868899481324</v>
       </c>
       <c r="D7" t="n">
-        <v>1887961595.389339</v>
+        <v>1965097203.315662</v>
       </c>
       <c r="E7" t="n">
-        <v>7.872273842718261e-12</v>
+        <v>7.324846663579629e-12</v>
       </c>
       <c r="F7" t="n">
-        <v>64.28571428571428</v>
+        <v>92.5</v>
       </c>
       <c r="G7" t="n">
-        <v>0.2900828473447833</v>
+        <v>0.2750544998927322</v>
       </c>
       <c r="H7" t="n">
         <v>0.2320005356687789</v>
       </c>
       <c r="I7" t="n">
-        <v>42.85714285714285</v>
+        <v>30</v>
       </c>
       <c r="J7" t="n">
-        <v>28.57142857142857</v>
+        <v>35</v>
       </c>
       <c r="K7" t="n">
-        <v>64.28571428571428</v>
+        <v>92.5</v>
       </c>
       <c r="L7" t="n">
-        <v>57.14285714285715</v>
+        <v>70</v>
       </c>
       <c r="M7" t="n">
-        <v>47.85714285714285</v>
+        <v>62.75</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>NEUTRO</t>
+          <t>COMPRA MODERADA</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>GGBR4</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.3891567935315539</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1.415164917480249</v>
+      </c>
+      <c r="D8" t="n">
+        <v>305083982.0285343</v>
+      </c>
+      <c r="E8" t="n">
+        <v>4.59382968532927e-11</v>
+      </c>
+      <c r="F8" t="n">
+        <v>50</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.2658475260538358</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.2356576570050664</v>
+      </c>
+      <c r="I8" t="n">
+        <v>15</v>
+      </c>
+      <c r="J8" t="n">
+        <v>55.00000000000001</v>
+      </c>
+      <c r="K8" t="n">
+        <v>50</v>
+      </c>
+      <c r="L8" t="n">
+        <v>85</v>
+      </c>
+      <c r="M8" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>COMPRA MODERADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.8723906410050846</v>
+      </c>
+      <c r="C9" t="n">
+        <v>2.795473343298629</v>
+      </c>
+      <c r="D9" t="n">
+        <v>672211787.9171462</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2.780498149560649e-11</v>
+      </c>
+      <c r="F9" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.3798624807423003</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.2996979632178868</v>
+      </c>
+      <c r="I9" t="n">
+        <v>70</v>
+      </c>
+      <c r="J9" t="n">
+        <v>75</v>
+      </c>
+      <c r="K9" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="L9" t="n">
+        <v>30</v>
+      </c>
+      <c r="M9" t="n">
+        <v>57.75</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>LREN3</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.4351572005999469</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1.178088442065718</v>
+      </c>
+      <c r="D10" t="n">
+        <v>214630220.641554</v>
+      </c>
+      <c r="E10" t="n">
+        <v>7.118133994725355e-11</v>
+      </c>
+      <c r="F10" t="n">
+        <v>45</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.2731148877027023</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.2950370246786932</v>
+      </c>
+      <c r="I10" t="n">
+        <v>25</v>
+      </c>
+      <c r="J10" t="n">
+        <v>45</v>
+      </c>
+      <c r="K10" t="n">
+        <v>45</v>
+      </c>
+      <c r="L10" t="n">
+        <v>75</v>
+      </c>
+      <c r="M10" t="n">
+        <v>54</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>B3SA3</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B11" t="n">
         <v>0.5652946993579147</v>
       </c>
-      <c r="C8" t="n">
-        <v>1.603692759145953</v>
-      </c>
-      <c r="D8" t="n">
-        <v>718105518.3993748</v>
-      </c>
-      <c r="E8" t="n">
-        <v>2.979485253428927e-11</v>
-      </c>
-      <c r="F8" t="n">
-        <v>14.28571428571428</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.391607290155775</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0.3268833044944129</v>
-      </c>
-      <c r="I8" t="n">
+      <c r="C11" t="n">
+        <v>1.60636460538609</v>
+      </c>
+      <c r="D11" t="n">
+        <v>735689106.6381091</v>
+      </c>
+      <c r="E11" t="n">
+        <v>2.648841306177606e-11</v>
+      </c>
+      <c r="F11" t="n">
+        <v>70</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.3848047824991799</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.326883304494413</v>
+      </c>
+      <c r="I11" t="n">
+        <v>75</v>
+      </c>
+      <c r="J11" t="n">
+        <v>60</v>
+      </c>
+      <c r="K11" t="n">
+        <v>70</v>
+      </c>
+      <c r="L11" t="n">
+        <v>25</v>
+      </c>
+      <c r="M11" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CMIG4</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.2073366268588333</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.9178408322187571</v>
+      </c>
+      <c r="D12" t="n">
+        <v>140328841.298512</v>
+      </c>
+      <c r="E12" t="n">
+        <v>9.300003725718047e-11</v>
+      </c>
+      <c r="F12" t="n">
+        <v>35</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.2730079963293071</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.2159653738419742</v>
+      </c>
+      <c r="I12" t="n">
+        <v>20</v>
+      </c>
+      <c r="J12" t="n">
+        <v>40</v>
+      </c>
+      <c r="K12" t="n">
+        <v>35</v>
+      </c>
+      <c r="L12" t="n">
+        <v>80</v>
+      </c>
+      <c r="M12" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>PETR3</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.1835250164673701</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.6735150016737629</v>
+      </c>
+      <c r="D13" t="n">
+        <v>548551949.2075239</v>
+      </c>
+      <c r="E13" t="n">
+        <v>2.897843747357004e-11</v>
+      </c>
+      <c r="F13" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.3043585734769</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.2480749195310926</v>
+      </c>
+      <c r="I13" t="n">
+        <v>40</v>
+      </c>
+      <c r="J13" t="n">
+        <v>20</v>
+      </c>
+      <c r="K13" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="L13" t="n">
+        <v>60</v>
+      </c>
+      <c r="M13" t="n">
+        <v>43.25</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>EGIE3</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.3173569035095156</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1.294946776151718</v>
+      </c>
+      <c r="D14" t="n">
+        <v>63415354.03135391</v>
+      </c>
+      <c r="E14" t="n">
+        <v>2.300490102629428e-10</v>
+      </c>
+      <c r="F14" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.2861116741962522</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.2282730427211578</v>
+      </c>
+      <c r="I14" t="n">
+        <v>35</v>
+      </c>
+      <c r="J14" t="n">
+        <v>50</v>
+      </c>
+      <c r="K14" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="L14" t="n">
+        <v>65</v>
+      </c>
+      <c r="M14" t="n">
+        <v>43.25</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SANB11</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.4734836304930192</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1.716616986122147</v>
+      </c>
+      <c r="D15" t="n">
+        <v>155228925.9065719</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1.665831753078481e-10</v>
+      </c>
+      <c r="F15" t="n">
+        <v>35</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.4669745848596029</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.3275497332138042</v>
+      </c>
+      <c r="I15" t="n">
+        <v>85</v>
+      </c>
+      <c r="J15" t="n">
+        <v>70</v>
+      </c>
+      <c r="K15" t="n">
+        <v>35</v>
+      </c>
+      <c r="L15" t="n">
+        <v>15</v>
+      </c>
+      <c r="M15" t="n">
+        <v>43</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1.657440006545143</v>
+      </c>
+      <c r="C16" t="n">
+        <v>4.40992991951932</v>
+      </c>
+      <c r="D16" t="n">
+        <v>31126376.16107577</v>
+      </c>
+      <c r="E16" t="n">
+        <v>7.590553192987411e-10</v>
+      </c>
+      <c r="F16" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.562923499652882</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.4015815611518613</v>
+      </c>
+      <c r="I16" t="n">
+        <v>95</v>
+      </c>
+      <c r="J16" t="n">
         <v>100</v>
       </c>
-      <c r="J8" t="n">
-        <v>42.85714285714285</v>
-      </c>
-      <c r="K8" t="n">
-        <v>14.28571428571428</v>
-      </c>
-      <c r="L8" t="n">
+      <c r="K16" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="L16" t="n">
+        <v>5</v>
+      </c>
+      <c r="M16" t="n">
+        <v>42.25</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>-0.05259838402796235</v>
+      </c>
+      <c r="C17" t="n">
+        <v>-0.1793372011702252</v>
+      </c>
+      <c r="D17" t="n">
+        <v>945156962.9523141</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1.878604030643424e-11</v>
+      </c>
+      <c r="F17" t="n">
+        <v>80</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.3383418151527141</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.3109067758927472</v>
+      </c>
+      <c r="I17" t="n">
+        <v>60</v>
+      </c>
+      <c r="J17" t="n">
+        <v>5</v>
+      </c>
+      <c r="K17" t="n">
+        <v>80</v>
+      </c>
+      <c r="L17" t="n">
+        <v>40</v>
+      </c>
+      <c r="M17" t="n">
+        <v>38</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>EVITAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0.3440992444295181</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.7767610250646355</v>
+      </c>
+      <c r="D18" t="n">
+        <v>92180799.61228144</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1.956183780587861e-10</v>
+      </c>
+      <c r="F18" t="n">
+        <v>20</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.3313297017178391</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.335042310596612</v>
+      </c>
+      <c r="I18" t="n">
+        <v>55.00000000000001</v>
+      </c>
+      <c r="J18" t="n">
+        <v>30</v>
+      </c>
+      <c r="K18" t="n">
+        <v>20</v>
+      </c>
+      <c r="L18" t="n">
+        <v>44.99999999999999</v>
+      </c>
+      <c r="M18" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>EVITAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.4455812064768776</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.7190918507700694</v>
+      </c>
+      <c r="D19" t="n">
+        <v>185846133.9653197</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1.710234443284166e-10</v>
+      </c>
+      <c r="F19" t="n">
+        <v>35</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.6594759159479772</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.5047893061829969</v>
+      </c>
+      <c r="I19" t="n">
+        <v>100</v>
+      </c>
+      <c r="J19" t="n">
+        <v>25</v>
+      </c>
+      <c r="K19" t="n">
+        <v>35</v>
+      </c>
+      <c r="L19" t="n">
         <v>0</v>
       </c>
-      <c r="M8" t="n">
-        <v>21.42857142857143</v>
-      </c>
-      <c r="N8" t="inlineStr">
+      <c r="M19" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="N19" t="inlineStr">
         <is>
           <t>EVITAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0.2035293579101562</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.4320579438463107</v>
+      </c>
+      <c r="D20" t="n">
+        <v>123911418.4472425</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1.947787954523034e-10</v>
+      </c>
+      <c r="F20" t="n">
+        <v>25</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.525996820518986</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.3997199290124713</v>
+      </c>
+      <c r="I20" t="n">
+        <v>90</v>
+      </c>
+      <c r="J20" t="n">
+        <v>15</v>
+      </c>
+      <c r="K20" t="n">
+        <v>25</v>
+      </c>
+      <c r="L20" t="n">
+        <v>10</v>
+      </c>
+      <c r="M20" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>VENDA FORTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>AZZA3</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0.08771372351520745</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.1769720545322384</v>
+      </c>
+      <c r="D21" t="n">
+        <v>74300549.18361846</v>
+      </c>
+      <c r="E21" t="n">
+        <v>2.552598163620268e-10</v>
+      </c>
+      <c r="F21" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.3897914426792795</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.3599359751696338</v>
+      </c>
+      <c r="I21" t="n">
+        <v>80</v>
+      </c>
+      <c r="J21" t="n">
+        <v>10</v>
+      </c>
+      <c r="K21" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="L21" t="n">
+        <v>20</v>
+      </c>
+      <c r="M21" t="n">
+        <v>13.75</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>VENDA FORTE</t>
         </is>
       </c>
     </row>
@@ -851,7 +1475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -874,92 +1498,261 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BBDC4</t>
+          <t>ALPA4</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.9977540622750996</v>
+        <v>1.657440006545143</v>
       </c>
       <c r="C2" t="n">
-        <v>3.524412195831653</v>
+        <v>4.40992991951932</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>VALE3</t>
+          <t>BBDC4</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.8207620043812851</v>
+        <v>0.9977540622750996</v>
       </c>
       <c r="C3" t="n">
-        <v>3.326412780089652</v>
+        <v>3.523123972571357</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ITUB4</t>
+          <t>NEOE3</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.6897098437509033</v>
+        <v>0.7674675202273207</v>
       </c>
       <c r="C4" t="n">
-        <v>3.147924644483759</v>
+        <v>3.430425306946491</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ABEV3</t>
+          <t>VALE3</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.3611223549013032</v>
+        <v>0.8207620043812851</v>
       </c>
       <c r="C5" t="n">
-        <v>1.694658525640141</v>
+        <v>3.315576634856987</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>B3SA3</t>
+          <t>ITUB4</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.5652946993579147</v>
+        <v>0.6897098437509033</v>
       </c>
       <c r="C6" t="n">
-        <v>1.603692759145953</v>
+        <v>3.142741731706303</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PETR4</t>
+          <t>BPAC11</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.2069384299168635</v>
+        <v>0.8723906410050846</v>
       </c>
       <c r="C7" t="n">
-        <v>0.8486515303908404</v>
+        <v>2.795473343298629</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>SANB11</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-0.002795726117860386</v>
+        <v>0.4734836304930192</v>
       </c>
       <c r="C8" t="n">
-        <v>-0.01056761352176577</v>
+        <v>1.716616986122147</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ABEV3</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.3611223549013032</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1.69311549253637</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>B3SA3</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.5652946993579147</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1.60636460538609</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>GGBR4</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.3891567935315539</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1.415164917480249</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>EGIE3</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.3173569035095156</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1.294946776151718</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>LREN3</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.4351572005999469</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1.178088442065718</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CMIG4</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.2073366268588333</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.9178408322187571</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PETR4</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.2069382818126475</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.8539868899481324</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.3440992444295181</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.7767610250646355</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.4455812064768776</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.7190918507700694</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>PETR3</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0.1835250164673701</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.6735150016737629</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.2035293579101562</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.4320579438463107</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>AZZA3</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0.08771372351520745</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.1769720545322384</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>-0.05259838402796235</v>
+      </c>
+      <c r="C21" t="n">
+        <v>-0.1793372011702252</v>
       </c>
     </row>
   </sheetData>
@@ -973,7 +1766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1001,65 +1794,65 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>VALE3</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>14768618124.3547</v>
+        <v>2462520192.389824</v>
       </c>
       <c r="C2" t="n">
-        <v>7.794816665266045e-13</v>
+        <v>7.219603890928269e-12</v>
       </c>
       <c r="D2" t="n">
-        <v>92.85714285714286</v>
+        <v>97.5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>VALE3</t>
+          <t>PETR4</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2398868387.076423</v>
+        <v>1965097203.315662</v>
       </c>
       <c r="C3" t="n">
-        <v>7.647041598128165e-12</v>
+        <v>7.324846663579629e-12</v>
       </c>
       <c r="D3" t="n">
-        <v>78.57142857142857</v>
+        <v>92.5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PETR4</t>
+          <t>ITUB4</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1887961595.389339</v>
+        <v>1720748464.992015</v>
       </c>
       <c r="C4" t="n">
-        <v>7.872273842718261e-12</v>
+        <v>9.931335673099017e-12</v>
       </c>
       <c r="D4" t="n">
-        <v>64.28571428571428</v>
+        <v>87.5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ITUB4</t>
+          <t>BBAS3</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1686611723.969523</v>
+        <v>945156962.9523141</v>
       </c>
       <c r="C5" t="n">
-        <v>1.00673188090829e-11</v>
+        <v>1.878604030643424e-11</v>
       </c>
       <c r="D5" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6">
@@ -1069,45 +1862,253 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>912551371.7137746</v>
+        <v>936702989.6828333</v>
       </c>
       <c r="C6" t="n">
-        <v>1.777495030877855e-11</v>
+        <v>1.602628234031397e-11</v>
       </c>
       <c r="D6" t="n">
-        <v>35.71428571428571</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ABEV3</t>
+          <t>B3SA3</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>444647890.4039565</v>
+        <v>735689106.6381091</v>
       </c>
       <c r="C7" t="n">
-        <v>2.519363398876523e-11</v>
+        <v>2.648841306177606e-11</v>
       </c>
       <c r="D7" t="n">
-        <v>14.28571428571429</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>B3SA3</t>
+          <t>ABEV3</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>718105518.3993748</v>
+        <v>451478543.6449369</v>
       </c>
       <c r="C8" t="n">
-        <v>2.979485253428927e-11</v>
+        <v>2.610922385939225e-11</v>
       </c>
       <c r="D8" t="n">
-        <v>14.28571428571428</v>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>672211787.9171462</v>
+      </c>
+      <c r="C9" t="n">
+        <v>2.780498149560649e-11</v>
+      </c>
+      <c r="D9" t="n">
+        <v>62.5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>PETR3</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>548551949.2075239</v>
+      </c>
+      <c r="C10" t="n">
+        <v>2.897843747357004e-11</v>
+      </c>
+      <c r="D10" t="n">
+        <v>57.5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>GGBR4</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>305083982.0285343</v>
+      </c>
+      <c r="C11" t="n">
+        <v>4.59382968532927e-11</v>
+      </c>
+      <c r="D11" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>LREN3</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>214630220.641554</v>
+      </c>
+      <c r="C12" t="n">
+        <v>7.118133994725355e-11</v>
+      </c>
+      <c r="D12" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>185846133.9653197</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1.710234443284166e-10</v>
+      </c>
+      <c r="D13" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SANB11</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>155228925.9065719</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1.665831753078481e-10</v>
+      </c>
+      <c r="D14" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CMIG4</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>140328841.298512</v>
+      </c>
+      <c r="C15" t="n">
+        <v>9.300003725718047e-11</v>
+      </c>
+      <c r="D15" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>NEOE3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>55593558.19838388</v>
+      </c>
+      <c r="C16" t="n">
+        <v>2.730831357123434e-11</v>
+      </c>
+      <c r="D16" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>123911418.4472425</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1.947787954523034e-10</v>
+      </c>
+      <c r="D17" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>92180799.61228144</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1.956183780587861e-10</v>
+      </c>
+      <c r="D18" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>AZZA3</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>74300549.18361846</v>
+      </c>
+      <c r="C19" t="n">
+        <v>2.552598163620268e-10</v>
+      </c>
+      <c r="D19" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>EGIE3</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>63415354.03135391</v>
+      </c>
+      <c r="C20" t="n">
+        <v>2.300490102629428e-10</v>
+      </c>
+      <c r="D20" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>31126376.16107577</v>
+      </c>
+      <c r="C21" t="n">
+        <v>7.590553192987411e-10</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2.5</v>
       </c>
     </row>
   </sheetData>
@@ -1121,7 +2122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1149,17 +2150,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>NEOE3</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.2541466886367213</v>
+        <v>0.01860445309896535</v>
       </c>
       <c r="C2" t="n">
-        <v>0.2151546327929952</v>
+        <v>0.02885617245514972</v>
       </c>
       <c r="D2" t="n">
-        <v>14.28571428571428</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -1169,92 +2170,300 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.260145169409522</v>
+        <v>0.2621068729596222</v>
       </c>
       <c r="C3" t="n">
-        <v>0.2301036255099778</v>
+        <v>0.2309923257263864</v>
       </c>
       <c r="D3" t="n">
-        <v>28.57142857142857</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PETR4</t>
+          <t>GGBR4</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.2900828473447833</v>
+        <v>0.2658475260538358</v>
       </c>
       <c r="C4" t="n">
-        <v>0.2320005356687789</v>
+        <v>0.2356576570050664</v>
       </c>
       <c r="D4" t="n">
-        <v>42.85714285714285</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BBDC4</t>
+          <t>CMIG4</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.3070159486932991</v>
+        <v>0.2730079963293071</v>
       </c>
       <c r="C5" t="n">
-        <v>0.2864134091531322</v>
+        <v>0.2159653738419742</v>
       </c>
       <c r="D5" t="n">
-        <v>57.14285714285714</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ITUB4</t>
+          <t>LREN3</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3252733872921393</v>
+        <v>0.2731148877027023</v>
       </c>
       <c r="C6" t="n">
-        <v>0.2523599946119469</v>
+        <v>0.2950370246786932</v>
       </c>
       <c r="D6" t="n">
-        <v>71.42857142857143</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>VALE3</t>
+          <t>PETR4</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.3567095385327261</v>
+        <v>0.2750544998927322</v>
       </c>
       <c r="C7" t="n">
-        <v>0.2543366296571614</v>
+        <v>0.2320005356687789</v>
       </c>
       <c r="D7" t="n">
-        <v>85.71428571428571</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>EGIE3</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.2861116741962522</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.2282730427211578</v>
+      </c>
+      <c r="D8" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>PETR3</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.3043585734769</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.2480749195310926</v>
+      </c>
+      <c r="D9" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BBDC4</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.3082365131172478</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.2864134091531322</v>
+      </c>
+      <c r="D10" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ITUB4</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.3283468072948462</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.2524664077859532</v>
+      </c>
+      <c r="D11" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BEEF3</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.3313297017178391</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.335042310596612</v>
+      </c>
+      <c r="D12" t="n">
+        <v>55.00000000000001</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BBAS3</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.3383418151527141</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.3109067758927472</v>
+      </c>
+      <c r="D13" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>VALE3</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.3639053817002734</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.2579701008656878</v>
+      </c>
+      <c r="D14" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>BPAC11</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.3798624807423003</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.2996979632178868</v>
+      </c>
+      <c r="D15" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>B3SA3</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>0.391607290155775</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0.3268833044944129</v>
-      </c>
-      <c r="D8" t="n">
+      <c r="B16" t="n">
+        <v>0.3848047824991799</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.326883304494413</v>
+      </c>
+      <c r="D16" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>AZZA3</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.3897914426792795</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.3599359751696338</v>
+      </c>
+      <c r="D17" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SANB11</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0.4669745848596029</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.3275497332138042</v>
+      </c>
+      <c r="D18" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>CSNA3</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.525996820518986</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.3997199290124713</v>
+      </c>
+      <c r="D19" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ALPA4</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0.562923499652882</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.4015815611518613</v>
+      </c>
+      <c r="D20" t="n">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>MGLU3</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0.6594759159479772</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.5047893061829969</v>
+      </c>
+      <c r="D21" t="n">
         <v>100</v>
       </c>
     </row>
@@ -1292,7 +2501,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>51.98%</t>
+          <t>49.87%</t>
         </is>
       </c>
     </row>
@@ -1304,7 +2513,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>R$ 3259.6M</t>
+          <t>R$ 594.0M</t>
         </is>
       </c>
     </row>
@@ -1316,7 +2525,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>31.21%</t>
+          <t>34.99%</t>
         </is>
       </c>
     </row>
@@ -1327,7 +2536,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>7</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
@@ -1338,7 +2547,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-03-09 20:03</t>
+          <t>2026-03-09 21:20</t>
         </is>
       </c>
     </row>

</xml_diff>